<commit_message>
add: add all (#3)
</commit_message>
<xml_diff>
--- a/Project/data/Data-Figure1/Summary.xlsx
+++ b/Project/data/Data-Figure1/Summary.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10313"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856AC6F9-D22F-8640-ABC9-E8410BEC3C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD34328-73DB-A343-A52F-436571036B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -750,6 +750,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="487069168"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>

</xml_diff>